<commit_message>
6차 배치 잔여 11곳 사용자 스크린샷으로 최종 확정 (101,105,110,119,132,147,153,155,157,166,169)
주요 정정:
- 153 한국도로공사: 명칭 정정(디지털본부→AI디지털본부), 하위부서 확정(AX혁신처·AI데이터처·디지털관리처·정보보안센터), CISO 확정
- 157 한국디자인진흥원: AX사업실 산하 보안전략팀 신규 발견(CISO 확정)
- 132 한국관세정보원: 연구교육센터 존속 재확인
- 나머지 8곳: 기존 기록과 일치 확인

165 한국문화진흥주식회사는 사용자 요청으로 보류

build_site.py + build_xlsx_274.py 재빌드 — 이로써 1~180번(1~6차) 전체 라이브 재검증 완결

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IT조직_비교표_공공기관274.xlsx
+++ b/IT조직_비교표_공공기관274.xlsx
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>디지털본부 (디지털전환·AI·데이터·모빌리티 혁신 총괄) — 통칭 'AI 디지털본부'</t>
+          <t>AI디지털본부</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>디지털본부 산하: 디지털계획처(디지털전환 기획), AI데이터처(AI·데이터 총괄, 하위 데이터품질부 등), 모빌리티 혁신 부서 — 정보보안 부서 별도 운영</t>
+          <t>AI디지털본부 산하: AX혁신처, AI데이터처, 디지털관리처, 정보보안센터</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>정보보안 담당부서 운영 — 전담 CISO 직제 확인불가</t>
+          <t>정보보안센터 (AI디지털본부 산하)</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr">
@@ -16381,7 +16381,7 @@
       </c>
       <c r="M212" s="3" t="inlineStr">
         <is>
-          <t>확인불가 (정보보안 업무는 AX사업팀 및 경영본부 경영지원실 자산안전팀 분담)</t>
+          <t>AX사업실 산하 '보안전략팀' (신규 확인). 경영본부 경영지원실 자산안전팀도 일부 분담</t>
         </is>
       </c>
       <c r="N212" s="3" t="inlineStr">

</xml_diff>